<commit_message>
Add Disallowed GST, MAF and MAF Plus funding streams
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01 Global Budget Paper/Annex B1 - NUHS FY25 operating subv by funding streams - Mock.xlsx
+++ b/01 Global Budget Paper/Annex B1 - NUHS FY25 operating subv by funding streams - Mock.xlsx
@@ -358,7 +358,7 @@
       </c>
       <c r="F9" t="inlineStr" s="7">
         <is>
-          <t xml:space="preserve">Mock Funding Programme 002</t>
+          <t xml:space="preserve">Disallowed Input Goods &amp; Services Tax (DiGST) Subvention</t>
         </is>
       </c>
       <c r="G9" s="9">
@@ -414,7 +414,7 @@
       </c>
       <c r="F10" t="inlineStr" s="7">
         <is>
-          <t xml:space="preserve">Mock Funding Programme 003</t>
+          <t xml:space="preserve">Medication Assistance Fund (MAF)</t>
         </is>
       </c>
       <c r="G10" s="9">
@@ -476,7 +476,7 @@
       </c>
       <c r="F11" t="inlineStr" s="7">
         <is>
-          <t xml:space="preserve">Mock Funding Programme 004</t>
+          <t xml:space="preserve">Medication Assistance Fund (MAF) Plus</t>
         </is>
       </c>
       <c r="G11" s="9">

</xml_diff>